<commit_message>
Update documentation and enhance Pipe class functionality
- Updated version number from 0.1.7 to 0.1.8 in configuration files.
- Enhanced `Pipe` class in `linepipe_tools.py` with additional methods for calculating outer diameter to wall thickness ratio, mid diameter, inner diameter, outer wall radius, and total coating thickness.
- Added methods for calculating equivalent coating density, steel weight, coating weights, total coating weight, content weight, water displaced weight, and submerged weight.
- Improved docstrings for clarity and added examples for new methods.
- Updated `example_1_pysubsea.py` to include coating thickness in data processing.
- Modified CSS for better visual distinction of method groups in documentation.
- Updated output CSV with new values for total outer diameter and vertical bearing capacity arrays.
</commit_message>
<xml_diff>
--- a/examples/example_1_output.xlsx
+++ b/examples/example_1_output.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_Github\py-subsea\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{BF4687C6-718F-46EE-B5CF-7854BF4D3103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1B00C0-EC43-4D3C-9B1F-B7EBB41785A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6375" yWindow="840" windowWidth="37830" windowHeight="19770" xr2:uid="{199D21A4-EDD8-4223-A9B9-642FCF4DBD78}"/>
+    <workbookView xWindow="20505" yWindow="1695" windowWidth="17385" windowHeight="18015" xr2:uid="{199D21A4-EDD8-4223-A9B9-642FCF4DBD78}"/>
   </bookViews>
   <sheets>
     <sheet name="example_1_output" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
   <si>
     <t>Sensitivity1</t>
   </si>
@@ -115,26 +115,10 @@
     <t>Vertical Bearing Capacity Arrays</t>
   </si>
   <si>
-    <t>[    0.           848.93102754  1199.08122637 ... 26255.33673193
- 26258.60613667 26261.87553182]</t>
-  </si>
-  <si>
-    <t>[    0.           924.87980385  1306.788781   ... 31084.11324326
- 31087.99819615 31091.88313548]</t>
-  </si>
-  <si>
     <t>Depth Arrays Model 2</t>
   </si>
   <si>
     <t>Vertical Bearing Capacity Arrays Model 2</t>
-  </si>
-  <si>
-    <t>[    0.           888.76176266  1257.40644829 ... 45079.6289539
- 45086.96614465 45094.30342012]</t>
-  </si>
-  <si>
-    <t>[    0.           967.89891021  1369.36861044 ... 51772.49473315
- 51780.94497238 51789.3953079 ]</t>
   </si>
   <si>
     <t>Lateral Friction Factor - Mean</t>
@@ -194,7 +178,20 @@
     <t>Lateral Friction Factor - R²</t>
   </si>
   <si>
-    <t>Parameters</t>
+    <t>[    0.           858.25022125  1212.29859501 ... 26826.57106063
+ 26829.91304534 26833.25502002]</t>
+  </si>
+  <si>
+    <t>[    0.           933.44358154  1318.93229098 ... 31653.29051462
+ 31657.24832575 31661.2061228 ]</t>
+  </si>
+  <si>
+    <t>[    0.           898.47176125  1271.14402315 ... 45880.91341458
+ 45888.38365077 45895.85397307]</t>
+  </si>
+  <si>
+    <t>[    0.           976.82257109  1381.993684   ... 52550.21769167
+ 52558.7975221  52567.37745017]</t>
   </si>
 </sst>
 </file>
@@ -202,8 +199,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="0.000E+00"/>
-    <numFmt numFmtId="170" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.000E+00"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -725,7 +722,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -750,22 +747,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1141,7 +1137,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2C43A9A-A907-42B3-A51E-311BCAB338C7}">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.28515625" bestFit="1" customWidth="1"/>
@@ -1149,9 +1145,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>55</v>
-      </c>
+      <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1420,7 +1414,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>20</v>
       </c>
@@ -1437,7 +1431,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>21</v>
       </c>
@@ -1454,7 +1448,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>25</v>
       </c>
@@ -1471,24 +1465,24 @@
         <v>1.29E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B20" s="9">
-        <v>0.27310000000000001</v>
+        <v>0.27910000000000001</v>
       </c>
       <c r="C20" s="9">
-        <v>0.32390000000000002</v>
+        <v>0.32990000000000003</v>
       </c>
       <c r="D20" s="9">
-        <v>0.27310000000000001</v>
+        <v>0.27910000000000001</v>
       </c>
       <c r="E20" s="9">
-        <v>0.32390000000000002</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.32990000000000003</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>27</v>
       </c>
@@ -1505,7 +1499,7 @@
         <v>32645871.838504601</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>28</v>
       </c>
@@ -1522,34 +1516,32 @@
         <v>29</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G22" s="15"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B23" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G23" s="15"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>29</v>
@@ -1564,34 +1556,32 @@
         <v>29</v>
       </c>
       <c r="F24" s="13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="G24" s="15"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>35</v>
-      </c>
       <c r="C25" s="11" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G25" s="15"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B26" s="12">
         <v>0.48421976839050601</v>
@@ -1606,11 +1596,10 @@
         <v>0.48421976839050601</v>
       </c>
       <c r="F26" s="14"/>
-      <c r="G26" s="15"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B27" s="12">
         <v>0.15019865261634999</v>
@@ -1625,11 +1614,10 @@
         <v>0.15019865261634999</v>
       </c>
       <c r="F27" s="14"/>
-      <c r="G27" s="15"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B28" s="12">
         <v>-0.77114850726020401</v>
@@ -1644,11 +1632,10 @@
         <v>-0.77114850726020401</v>
       </c>
       <c r="F28" s="14"/>
-      <c r="G28" s="15"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B29" s="12">
         <v>0.303091071660128</v>
@@ -1663,11 +1650,10 @@
         <v>0.303091071660128</v>
       </c>
       <c r="F29" s="14"/>
-      <c r="G29" s="15"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B30" s="12">
         <v>0.28091898641840501</v>
@@ -1682,11 +1668,10 @@
         <v>0.28091898641840501</v>
       </c>
       <c r="F30" s="14"/>
-      <c r="G30" s="15"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B31" s="12">
         <v>0.462481599696904</v>
@@ -1701,11 +1686,10 @@
         <v>0.462481599696904</v>
       </c>
       <c r="F31" s="14"/>
-      <c r="G31" s="15"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B32" s="12">
         <v>0.76139114975887601</v>
@@ -1720,11 +1704,10 @@
         <v>0.76139114975887601</v>
       </c>
       <c r="F32" s="14"/>
-      <c r="G32" s="15"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B33" s="12">
         <v>2.8829223456266199E-2</v>
@@ -1739,11 +1722,10 @@
         <v>2.8829223456266199E-2</v>
       </c>
       <c r="F33" s="14"/>
-      <c r="G33" s="15"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B34" s="12">
         <v>0.980053020997808</v>
@@ -1758,49 +1740,46 @@
         <v>0.980053020997808</v>
       </c>
       <c r="F34" s="14"/>
-      <c r="G34" s="15"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B36" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C35" s="11" t="s">
+      <c r="C36" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D35" s="11" t="s">
+      <c r="D36" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E35" s="11" t="s">
+      <c r="E36" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F35" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G35" s="15"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
+      <c r="F36" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="C36" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="E36" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="F36" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G36" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>